<commit_message>
Update strategy benchmark analysis spreadsheet and remove temporary file
</commit_message>
<xml_diff>
--- a/environment/2d-environment/starter-stack/strategy_benchmark_analysis.xlsx
+++ b/environment/2d-environment/starter-stack/strategy_benchmark_analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan.sidib/Code/ENG5325-Robotics-TDP-M-Team-14/Cyberphysical-RoboCup-Soccer-Teams/environment/2d-environment/starter-stack/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F4E025CC-B773-C64A-B7D0-A14BBAC9EFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F91A4B-B77D-DA4A-9D14-E18F8DF94339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{5BADAF71-6070-6942-999C-7247CF5927ED}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{5BADAF71-6070-6942-999C-7247CF5927ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>